<commit_message>
Rebuild all Section 1-3 answer workbooks to the current questions
Thirty-one workbooks rewritten in place over their existing SharePoint
files so every share link and embed keeps working: Section 1 in-sheet
answers with per-part colour highlights and legends; Sections 2-3 with
a Data sheet (the filtered column or full dataset) and a formula
Answer sheet with written explanations. Four new embeds wired for the
questions that lacked workbooks; Peter's deletion of the XLOOKUP
question absorbed and numbering closed back to 42.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TNVxQFJXojPDm4Z5hNnmdq
</commit_message>
<xml_diff>
--- a/practice/answers/s1_q01.xlsx
+++ b/practice/answers/s1_q01.xlsx
@@ -16,10 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="$#,##0"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -33,7 +32,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -60,11 +59,6 @@
         <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D2E9"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -78,34 +72,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,18 +452,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -501,27 +480,24 @@
           <t>Yield (bu/ac)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Revenue ($/ac)</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Total revenue ($)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Bushels</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Canola price ($/bu)</t>
-        </is>
-      </c>
-      <c r="G1" s="20" t="n">
-        <v>14.2</v>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>Incorrect (no $ signs)</t>
         </is>
       </c>
     </row>
@@ -531,28 +507,26 @@
           <t>Kestrel</t>
         </is>
       </c>
-      <c r="B2" s="6" t="n">
+      <c r="B2" t="n">
         <v>120</v>
       </c>
-      <c r="C2" s="21" t="n">
+      <c r="C2" t="n">
         <v>41.2</v>
       </c>
-      <c r="D2" s="22">
-        <f>C2*$G$1</f>
-        <v/>
-      </c>
-      <c r="E2" s="9">
+      <c r="D2" s="2">
+        <f>C2*$H$2</f>
+        <v/>
+      </c>
+      <c r="E2" s="3">
         <f>D2*B2</f>
         <v/>
       </c>
-      <c r="H2" s="23">
-        <f>C2*G1</f>
-        <v/>
-      </c>
-      <c r="I2" s="11" t="inlineStr">
-        <is>
-          <t>Only the first row is right; the rows below show $0.00 because the unanchored price reference walks down to G2, G3, ... which are empty and treated as zero.</t>
-        </is>
+      <c r="F2" s="4">
+        <f>B2*C2</f>
+        <v/>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>14.2</v>
       </c>
     </row>
     <row r="3">
@@ -561,25 +535,24 @@
           <t>Meadowvale</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" t="n">
         <v>240</v>
       </c>
-      <c r="C3" s="21" t="n">
+      <c r="C3" t="n">
         <v>38.6</v>
       </c>
-      <c r="D3" s="22">
-        <f>C3*$G$1</f>
-        <v/>
-      </c>
-      <c r="E3" s="9">
+      <c r="D3" s="2">
+        <f>C3*$H$2</f>
+        <v/>
+      </c>
+      <c r="E3" s="3">
         <f>D3*B3</f>
         <v/>
       </c>
-      <c r="H3" s="23">
-        <f>C3*G2</f>
-        <v/>
-      </c>
-      <c r="I3" s="19" t="n"/>
+      <c r="F3" s="4">
+        <f>B3*C3</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -587,25 +560,24 @@
           <t>Nightjar</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" t="n">
         <v>95</v>
       </c>
-      <c r="C4" s="21" t="n">
+      <c r="C4" t="n">
         <v>44.8</v>
       </c>
-      <c r="D4" s="22">
-        <f>C4*$G$1</f>
-        <v/>
-      </c>
-      <c r="E4" s="9">
+      <c r="D4" s="2">
+        <f>C4*$H$2</f>
+        <v/>
+      </c>
+      <c r="E4" s="3">
         <f>D4*B4</f>
         <v/>
       </c>
-      <c r="H4" s="23">
-        <f>C4*G3</f>
-        <v/>
-      </c>
-      <c r="I4" s="19" t="n"/>
+      <c r="F4" s="4">
+        <f>B4*C4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -613,25 +585,24 @@
           <t>Home</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" t="n">
         <v>310</v>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" t="n">
         <v>36.1</v>
       </c>
-      <c r="D5" s="22">
-        <f>C5*$G$1</f>
-        <v/>
-      </c>
-      <c r="E5" s="9">
+      <c r="D5" s="2">
+        <f>C5*$H$2</f>
+        <v/>
+      </c>
+      <c r="E5" s="3">
         <f>D5*B5</f>
         <v/>
       </c>
-      <c r="H5" s="23">
-        <f>C5*G4</f>
-        <v/>
-      </c>
-      <c r="I5" s="19" t="n"/>
+      <c r="F5" s="4">
+        <f>B5*C5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -639,97 +610,89 @@
           <t>Rented</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" t="n">
         <v>175</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" t="n">
         <v>39.9</v>
       </c>
-      <c r="D6" s="22">
-        <f>C6*$G$1</f>
-        <v/>
-      </c>
-      <c r="E6" s="9">
+      <c r="D6" s="2">
+        <f>C6*$H$2</f>
+        <v/>
+      </c>
+      <c r="E6" s="3">
         <f>D6*B6</f>
         <v/>
       </c>
-      <c r="H6" s="23">
-        <f>C6*G5</f>
-        <v/>
-      </c>
-      <c r="I6" s="19" t="n"/>
+      <c r="F6" s="4">
+        <f>B6*C6</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Total acres</t>
-        </is>
-      </c>
-      <c r="B8" s="13">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Totals (c)</t>
+        </is>
+      </c>
+      <c r="B8" s="4">
         <f>SUM(B2:B6)</f>
         <v/>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Total bushels</t>
-        </is>
-      </c>
-      <c r="B9" s="14">
-        <f>SUMPRODUCT(B2:B6,C2:C6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Total revenue ($)</t>
-        </is>
-      </c>
-      <c r="B10" s="24">
+      <c r="E8" s="6">
         <f>SUM(E2:E6)</f>
         <v/>
       </c>
+      <c r="F8" s="4">
+        <f>SUM(F2:F6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>(d) The price sits in one cell (H2), so as the part a formula fills down every copy must keep pointing at it -- the $ signs lock that reference. In part b, revenue per acre and acres both sit on the same row as the formula, so both references should shift down together and no $ is needed.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Legend: colours mark question parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Part (a)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Part (b)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Part (c)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Part (d)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>Part (e)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="I2:I6"/>
+    <mergeCell ref="A10:F10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>